<commit_message>
docs(capability): retain raw validation logs as .log.txt
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/evidence/integration/capability-matrix-51x17-reassessment-2026-10-31/IIPS_V3_CAPABILITY_MATRIX_51x17_REASSESSED_2026-10-31.xlsx
+++ b/evidence/integration/capability-matrix-51x17-reassessment-2026-10-31/IIPS_V3_CAPABILITY_MATRIX_51x17_REASSESSED_2026-10-31.xlsx
@@ -9390,7 +9390,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>raw/irr-test-ci.log; raw/irr-vitest-report.json; raw/irr-build.log</t>
+          <t>raw/irr-test-ci.log.txt; raw/irr-vitest-report.json; raw/irr-build.log.txt</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>raw/ipd-test.log; raw/ipd-typecheck.log; raw/ipd-package-consumer.log</t>
+          <t>raw/ipd-test.log.txt; raw/ipd-typecheck.log.txt; raw/ipd-package-consumer.log.txt</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(cap03): resolve P-11/P-18/P-19/P-20 and assess G14 dependencies
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/evidence/integration/capability-matrix-51x17-reassessment-2026-10-31/IIPS_V3_CAPABILITY_MATRIX_51x17_REASSESSED_2026-10-31.xlsx
+++ b/evidence/integration/capability-matrix-51x17-reassessment-2026-10-31/IIPS_V3_CAPABILITY_MATRIX_51x17_REASSESSED_2026-10-31.xlsx
@@ -16,9 +16,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Updated Capability Matrix'!$A$1:$Q$52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outstanding-Pending Items'!$A$1:$P$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reconciliation'!$A$1:$B$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Evidence Register'!$A$1:$F$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outstanding-Pending Items'!$A$1:$P$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reconciliation'!$A$1:$B$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Evidence Register'!$A$1:$F$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Branch-PR Census'!$A$1:$J$407</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Validation'!$A$1:$C$12</definedName>
   </definedNames>
@@ -240,8 +240,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PendingItems" displayName="PendingItems" ref="A1:P45" headerRowCount="1">
-  <autoFilter ref="A1:P45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PendingItems" displayName="PendingItems" ref="A1:P41" headerRowCount="1">
+  <autoFilter ref="A1:P41"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Item ID"/>
     <tableColumn id="2" name="Group"/>
@@ -265,8 +265,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Reconciliation" displayName="Reconciliation" ref="A1:B31" headerRowCount="1">
-  <autoFilter ref="A1:B31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Reconciliation" displayName="Reconciliation" ref="A1:B30" headerRowCount="1">
+  <autoFilter ref="A1:B30"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Value"/>
@@ -276,8 +276,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EvidenceRegister" displayName="EvidenceRegister" ref="A1:F37" headerRowCount="1">
-  <autoFilter ref="A1:F37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EvidenceRegister" displayName="EvidenceRegister" ref="A1:F43" headerRowCount="1">
+  <autoFilter ref="A1:F43"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Evidence ID"/>
     <tableColumn id="2" name="Repository"/>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; frontend/src/features/sector/**; /api/sector/banking 404 by design; PKG-08 row-4 acceptance [E006][E008]. Pending: P-01.</t>
+          <t>IRR main@fff8cf98; frontend/src/features/sector/**; /api/sector/banking 404 by design; PKG-08 row-4 acceptance [E006][E008]. P-01. Pending: P-01.</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; live GET /api/cross-sector 200 avgConviction 72.9; iips-cross-sector/CSIP_*; program-v1.1-certification [E006][E008]. Pending: P-02.</t>
+          <t>IRR main@fff8cf98; live GET /api/cross-sector 200 avgConviction 72.9; iips-cross-sector/CSIP_*; program-v1.1-certification [E006][E008]. P-02. Pending: P-02.</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; frontend/server/watchlists/**; restart block 15/15; GET /api/watchlists 503 [E006][E008]. Pending: P-03.</t>
+          <t>IRR main@fff8cf98; frontend/server/watchlists/**; restart block 15/15; GET /api/watchlists 503 [E006][E008]. P-03. Pending: P-03.</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; frontend/server/collaboration/**; restart block 15/15; GET /api/collaboration 503 [E006][E008]. Pending: P-03.</t>
+          <t>IRR main@fff8cf98; frontend/server/collaboration/**; restart block 15/15; GET /api/collaboration 503 [E006][E008]. P-03. Pending: P-03.</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; frontend/server/settings/**; restart block 15/15; GET /api/settings 503 [E006][E008]. Pending: P-03.</t>
+          <t>IRR main@fff8cf98; frontend/server/settings/**; restart block 15/15; GET /api/settings 503 [E006][E008]. P-03. Pending: P-03.</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; live GET /api/macro/NAS 502 RETRY_BUDGET_EXHAUSTED in sandbox; tracker §§16.29/16.31 live E2E A [E008][E027]. Pending: P-04, P-35.</t>
+          <t>IRR main@fff8cf98; live GET /api/macro/NAS 502 RETRY_BUDGET_EXHAUSTED in sandbox; tracker §§16.29/16.31 live E2E A [E008][E027]. P-04. Pending: P-04, P-35.</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; frontend/server/d115-runtime.ts; CV-43 retain-unwired disposition [E025]. Pending: P-05 (only if PA commissions wiring).</t>
+          <t>IRR main@fff8cf98; frontend/server/d115-runtime.ts; CV-43 retain-unwired disposition [E025]. P-05 (only if PA commissions wiring). Pending: P-05.</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>IPD main@4e275ec9; src/identity/security_master.ts; tests/d05_*; guarded suite 941/940/0/1 [E007]; no per-record REAL classification (SMI-01). Pending: P-30.</t>
+          <t>IPD main@4e275ec9; src/identity/security_master.ts; tests/d05_*; guarded suite 941/940/0/1 [E007]; no per-record REAL classification (SMI-01). P-30. Pending: P-30.</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>IPD main@4e275ec9; src/ui/**; tests/shell_*; guarded suite 941/940/0/1 [E007]; tracker §18 row 27 / O-09. Pending: P-06, P-34.</t>
+          <t>IPD main@4e275ec9; src/ui/**; tests/shell_*; guarded suite 941/940/0/1 [E007]; tracker §18 row 27 / O-09. P-06. Pending: P-06, P-34.</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>IPD main@4e275ec9; src/ipc/brokerImportConsumer.ts 308c83ee; src/ipc/entrypoint.ts 16d4112e; guard 540d49f2 authorized:false; IRR §16.227 [E014]. Pending: P-07, P-22, P-23, P-24, P-25, P-26, P-32, P-44.</t>
+          <t>IPD main@4e275ec9; src/ipc/brokerImportConsumer.ts 308c83ee; src/ipc/entrypoint.ts 16d4112e; guard 540d49f2 authorized:false; IRR §16.227 [E014]. P-07, P-22. Pending: P-07, P-22, P-23, P-24, P-25, P-26, P-32, P-44.</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>IPD main@4e275ec9; src/operator_drop/**; src/oq/synthetic_failover.ts; package.json exports; REG-06 deferred [E018][E026]. Pending: P-08.</t>
+          <t>IPD main@4e275ec9; src/operator_drop/**; src/oq/synthetic_failover.ts; package.json exports; REG-06 deferred [E018][E026]. P-08. Pending: P-08.</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; /api/user-portfolios* 503; tracker §16.229 S00 stop; P1-F act [E004][E008][E011]. Pending: P-09, P-10, P-11, P-21, P-22, P-23, P-24, P-25, P-26, P-27, P-28, P-29, P-31, P-32, P-34, P-36, P-37, P-38, P-39, P-40, P-42, P-43.</t>
+          <t>IRR main@fff8cf98; /api/user-portfolios* 503; tracker §16.229 S00 stop; P1-F act [E004][E008][E011]. P-09, P-10, P-11. Pending: P-09, P-10, P-21, P-22, P-23, P-24, P-25, P-26, P-27, P-28, P-29, P-31, P-32, P-34, P-36, P-37, P-38, P-39, P-40, P-42, P-43.</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; server/user-portfolio contract/port/boundary; portfolio/reports/broker-import block 24 files / 385 tests passed [E006]; D-2 §8 / G-2 §5. Pending: P-32.</t>
+          <t>IRR main@fff8cf98; server/user-portfolio contract/port/boundary; portfolio/reports/broker-import block 24 files / 385 tests passed [E006]; D-2 §8 / G-2 §5. P-32. Pending: P-32.</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>IRR full-clone census: arena/a2df3b85@5eba01b6 7 ahead / 920 behind; 470cc698 not ancestor; CV-52 [E009][E020]. Pending: P-12, P-09, P-10, P-21, P-22, P-23, P-24, P-25, P-27, P-28, P-29, P-38, P-39, P-40, P-42, P-43.</t>
+          <t>IRR full-clone census: arena/a2df3b85@5eba01b6 7 ahead / 920 behind; 470cc698 not ancestor; CV-52 [E009][E020]. P-12. Pending: P-09, P-10, P-12, P-21, P-22, P-23, P-24, P-25, P-27, P-28, P-29, P-38, P-39, P-40, P-42, P-43.</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; blobs reports-transport 775d282b, user-portfolio-transport 51704c12, owner-context-unavailable cb8db45d; live 503/404 probes [E006][E008]. Pending: P-31.</t>
+          <t>IRR main@fff8cf98; blobs reports-transport 775d282b, user-portfolio-transport 51704c12, owner-context-unavailable cb8db45d; live 503/404 probes [E006][E008]. P-31. Pending: P-31.</t>
         </is>
       </c>
     </row>
@@ -3690,7 +3690,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; frontend/server/reports/** 10 files; reports-transport 775d282b; F-7/CV-51 accepted bounded; D-9 CLOSED C4-2 [E006][E015]. Pending: P-13, P-41.</t>
+          <t>IRR main@fff8cf98; frontend/server/reports/** 10 files; reports-transport 775d282b; F-7/CV-51 accepted bounded; D-9 CLOSED C4-2 [E006][E015]. P-13. Pending: P-13, P-41.</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; resolveDataDir/IIPS_DATA_DIR; .gitignore; CV-24 F6/TD-7b reserved [E019]. Pending: P-14.</t>
+          <t>IRR main@fff8cf98; resolveDataDir/IIPS_DATA_DIR;.gitignore; CV-24 F6/TD-7b reserved [E019]. P-14. Pending: P-14.</t>
         </is>
       </c>
     </row>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; CV-22 Option C; screener memberCount 13 executed [E008][E017]. Pending: P-15, P-30.</t>
+          <t>IRR main@fff8cf98; CV-22 Option C; screener memberCount 13 executed [E008][E017]. P-15. Pending: P-15, P-30.</t>
         </is>
       </c>
     </row>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; frontend/package.json three pins; guard blobs 0a1e58de / 4f6024f0; O-06 closed §16.211 [E016][E024]. Pending: P-16, P-17, P-36.</t>
+          <t>IRR main@fff8cf98; frontend/package.json three pins; guard blobs 0a1e58de / 4f6024f0; O-06 closed §16.211 [E016][E024]. P-16, P-17. Pending: P-16, P-17, P-36.</t>
         </is>
       </c>
     </row>
@@ -4673,9 +4673,9 @@
           <t>V — documents the restart-proof commands; those commands were executed today.</t>
         </is>
       </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>P — start path and probes reproduced; runbook headline figures are stale: document says 106 files / 1350 tests, current head executes 108 / 1377 [E006][E023].</t>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>V — start path and probes reproduced; runbook restamped to 108 files / 1377 tests at exact frontend tree 67607e1d with raw receipts [E023][E039].</t>
         </is>
       </c>
       <c r="K48" s="4" t="inlineStr">
@@ -4703,14 +4703,14 @@
           <t>P — Linux qualification; Windows not claimed.</t>
         </is>
       </c>
-      <c r="P48" s="4" t="inlineStr">
-        <is>
-          <t>P — operator-facing readiness current except runbook figure restamp (P-18) [E023].</t>
+      <c r="P48" s="3" t="inlineStr">
+        <is>
+          <t>V — operator-facing readiness current for the verified non-production baseline; runbook restamp complete [E023][E039].</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>IRR main@fff8cf98; docs/OPERATOR_RUNBOOK.md e94d2b80; live start/probe; current suite 108/1377 [E006][E008][E023]. Pending: P-18.</t>
+          <t>IRR main@7fd824de; docs/OPERATOR_RUNBOOK.md restamped; live start/probe; current suite 108/1377 [E008][E023][E039]. P-18.</t>
         </is>
       </c>
     </row>
@@ -4725,7 +4725,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>V — master tracker at main@fff8cf98 through §16.229 (blob edf4fb64) + IPD cross-repository evidence set; dated overlays govern historical text [E004][E005].</t>
+          <t>V — master tracker at main@7fd824de through §16.232, with §16.233 consolidated resolution overlay; IPD cross-repository evidence set corrected by PR #114; dated overlays govern historical text [E004][E005][E041].</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -4790,12 +4790,12 @@
       </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>P — integrity good; open PR #398 proposes §16.230 and is not merged; IPD tracker footer P-1 status stale vs IRR P1-F (recorded conflict) [E005][E010].</t>
+          <t>P — tracker integrity good; PR #398 merged and IPD P-20 corrected; G14 final reconciliation remains blocked by upstream gates and P1-F consumption remains NOT RECONCILED [E010][E038][E040].</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>IRR tracker §§16.207/16.211/16.229; IPD tracker; PR #398 OPEN/UNSTABLE [E004][E005][E010][E016]. Pending: P-19, P-20, P-11, P-33, P-37, P-39.</t>
+          <t>IRR tracker §§16.207/16.211/16.229/16.230/16.232/16.233; IPD PR #114; PR #398 MERGED [E004][E005][E010][E016][E038][E041]. P-11, P-19, P-20, P-33. Pending: P-33, P-37, P-39.</t>
         </is>
       </c>
     </row>
@@ -5069,7 +5069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5995,206 +5995,206 @@
     <row r="12" ht="95" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>P-11</t>
+          <t>P-12</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>IRR implementation / deliverables</t>
+          <t>Cross-repository integration / dependencies</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,48 — Validation, Governance</t>
+          <t>Row 32 — Authority, Acceptance, Qualification</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>PR #398 consolidated P1/S2 correction</t>
+          <t>G24 branch-only lineage / CV-52 admission</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>OPEN — UNMERGED / Windows CI FAILURE</t>
+          <t>BLOCKED — branch-only, unadmitted</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Review, correct Windows PowerShell fixture failure, merge and read back PR #398; it proposes §16.230 and script/S2 artifact retention changes.</t>
+          <t>Obtain explicit CV-52 admission act naming qualified commits, or recorded permanent no; re-qualify if promoted.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Windows CI green + PA/owner review</t>
+          <t>Gate 4 qualification/acceptance + Gate 5 admission</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>IRR maintainer</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>IRR + IPD</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Ordinary IRR PR admission; no IPD write</t>
+          <t>CV-52 admission act</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Windows fixture run 41207888891 failed; static check passed</t>
+          <t>470cc698 not ancestor; branch 7 ahead / 920 behind</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Merged PR, green exact-head CI, remote blob read-back, tracker publication</t>
+          <t>Admission act + qualified commit identities + integration evidence</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>IRR PR #398 head e3dcb4d [E010]</t>
+          <t>IRR arena/a2df3b85@5eba01b6; CV-52 [E009][E020]</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Fix failing Windows fixture workflow and re-run checks</t>
+          <t>Do not promote branch by default; complete qualification/admission chain</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>PR merged with green checks; authoritative script identity updated; no host execution inferred</t>
+          <t>CV-52 admitted with named qualified commits or closed by recorded no</t>
         </is>
       </c>
     </row>
     <row r="13" ht="95" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>P-12</t>
+          <t>P-13</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Cross-repository integration / dependencies</t>
+          <t>Evidence / certification / verification</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Row 32 — Authority, Acceptance, Qualification</t>
+          <t>Row 35 — Release-readiness</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>G24 branch-only lineage / CV-52 admission</t>
+          <t>Reports G-14 operator network hardening evidence</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>BLOCKED — branch-only, unadmitted</t>
+          <t>OPEN — non-blocking residual</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Obtain explicit CV-52 admission act naming qualified commits, or recorded permanent no; re-qualify if promoted.</t>
+          <t>Evidence operator-side network hardening before any isolation claim or broader exposure; D-9 itself is closed.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Gate 4 qualification/acceptance + Gate 5 admission</t>
+          <t>Operator network evidence / separate act if exposure changes</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>IRR + IPD</t>
+          <t>Operator</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>CV-52 admission act</t>
+          <t>Separate authoritative act for isolation/broader exposure</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>470cc698 not ancestor; branch 7 ahead / 920 behind</t>
+          <t>Loopback binding evidenced in source; operator hardening unevidenced</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Admission act + qualified commit identities + integration evidence</t>
+          <t>Network posture evidence or explicit no-isolation-claim disposition</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>IRR arena/a2df3b85@5eba01b6; CV-52 [E009][E020]</t>
+          <t>IRR tracker §16.215.3 [E029]</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Do not promote branch by default; complete qualification/admission chain</t>
+          <t>Record residual; capture hardening evidence only if isolation claimed</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>CV-52 admitted with named qualified commits or closed by recorded no</t>
+          <t>G-14 evidenced or formally retained as no-isolation-claim boundary</t>
         </is>
       </c>
     </row>
     <row r="14" ht="95" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>P-13</t>
+          <t>P-14</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Evidence / certification / verification</t>
+          <t>PA decisions / governance</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Row 35 — Release-readiness</t>
+          <t>Row 39 — Authority, Acceptance</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Reports G-14 operator network hardening evidence</t>
+          <t>CV-24 F6 inventory / TD-7b production profile</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>OPEN — non-blocking residual</t>
+          <t>DECISION REQUIRED — non-blocking</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Evidence operator-side network hardening before any isolation claim or broader exposure; D-9 itself is closed.</t>
+          <t>PA decides F6_INVENTORY_AUTHORIZED yes/no and TD-7b production data-directory profile (including out-of-scope-for-non-production closure if chosen).</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Operator network evidence / separate act if exposure changes</t>
+          <t>PA decision</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Operator</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -6204,44 +6204,44 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Operator</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Separate authoritative act for isolation/broader exposure</t>
+          <t>One combined CV-24 act</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Loopback binding evidenced in source; operator hardening unevidenced</t>
+          <t>No current non-production blocker</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Network posture evidence or explicit no-isolation-claim disposition</t>
+          <t>Rendered act naming each disposition</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>IRR tracker §16.215.3 [E029]</t>
+          <t>IRR tracker CV-24 [E019]</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Record residual; capture hardening evidence only if isolation claimed</t>
+          <t>Put combined CV-24 decision to PA</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>G-14 evidenced or formally retained as no-isolation-claim boundary</t>
+          <t>Each named item has explicit disposition; no inferred production profile</t>
         </is>
       </c>
     </row>
     <row r="15" ht="95" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>P-14</t>
+          <t>P-15</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -6251,27 +6251,27 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Row 39 — Authority, Acceptance</t>
+          <t>Row 41 — Authority, Acceptance</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>CV-24 F6 inventory / TD-7b production profile</t>
+          <t>CV-22 governed-universe expansion</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>DECISION REQUIRED — non-blocking</t>
+          <t>DEFERRED — Option C</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>PA decides F6_INVENTORY_AUTHORIZED yes/no and TD-7b production data-directory profile (including out-of-scope-for-non-production closure if chosen).</t>
+          <t>Future expansion requires identity/eligibility contract, approved roster/corpus, exact mapping, consumer acceptance criteria and separate implementation authority.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>PA decision</t>
+          <t>Defined prerequisites + PA authority</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -6286,44 +6286,44 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>IRR + IPD</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>One combined CV-24 act</t>
+          <t>New PA expansion act</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>No current non-production blocker</t>
+          <t>13-row universe preserved; no REAL-only subset inferred</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Rendered act naming each disposition</t>
+          <t>Prerequisite package + PA act + consumer acceptance evidence</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>IRR tracker CV-24 [E019]</t>
+          <t>IRR CV-22 Option C [E017]</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Put combined CV-24 decision to PA</t>
+          <t>Preserve 13-row baseline; no expansion without prerequisites</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Each named item has explicit disposition; no inferred production profile</t>
+          <t>Expansion accepted with evidence or deferral retained</t>
         </is>
       </c>
     </row>
     <row r="16" ht="95" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>P-15</t>
+          <t>P-16</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -6333,79 +6333,79 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Row 41 — Authority, Acceptance</t>
+          <t>Row 45 — Release-readiness</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>CV-22 governed-universe expansion</t>
+          <t>DQ-4 final QE freeze</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>DEFERRED — Option C</t>
+          <t>NOT ESTABLISHED — 8/10</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Future expansion requires identity/eligibility contract, approved roster/corpus, exact mapping, consumer acceptance criteria and separate implementation authority.</t>
+          <t>Render DQ-4 freeze act after host sequence S2 → one P-1 → S3 and native-Windows canonical evidence; criteria 7-8 not met.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Defined prerequisites + PA authority</t>
+          <t>P-1 execution, S3, native evidence, final Gate 4 pin/H-12</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
+          <t>PA + operator</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>IRR + IPD</t>
+          <t>Operator</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>New PA expansion act</t>
+          <t>DQ-4 freeze act</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>13-row universe preserved; no REAL-only subset inferred</t>
+          <t>Host sequence unexecuted; no final freeze</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Prerequisite package + PA act + consumer acceptance evidence</t>
+          <t>Freeze act + criteria 7/8 evidence + remote read-back</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>IRR CV-22 Option C [E017]</t>
+          <t>IRR DQ-4 manifest; tracker §16.122.9/§16.123 [E013]</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>Preserve 13-row baseline; no expansion without prerequisites</t>
+          <t>Complete host sequence then freeze</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Expansion accepted with evidence or deferral retained</t>
+          <t>10/10 criteria met and freeze act effective; drift rule bound</t>
         </is>
       </c>
     </row>
     <row r="17" ht="95" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>P-16</t>
+          <t>P-17</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -6420,27 +6420,27 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>DQ-4 final QE freeze</t>
+          <t>Alias modernization / permanent pin architecture</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>NOT ESTABLISHED — 8/10</t>
+          <t>OPEN — NOT AUTHORIZED — OFF CRITICAL PATH</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Render DQ-4 freeze act after host sequence S2 → one P-1 → S3 and native-Windows canonical evidence; criteria 7-8 not met.</t>
+          <t>Only if PA commissions: B-1 governed IPD export or B-2 IRR broker-build redesign plus requalification tail; not an O-06 guard defect.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>P-1 execution, S3, native evidence, final Gate 4 pin/H-12</t>
+          <t>Separate PA act</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>PA + operator</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -6450,44 +6450,44 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Operator</t>
+          <t>IRR + IPD</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>DQ-4 freeze act</t>
+          <t>CAP03-DQ6B-FOLLOW-ON-ALIAS-MODERNIZATION authority</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Host sequence unexecuted; no final freeze</t>
+          <t>Interim guarded split is accepted; no current blocker</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Freeze act + criteria 7/8 evidence + remote read-back</t>
+          <t>PA act + scoped implementation + requalification evidence</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>IRR DQ-4 manifest; tracker §16.122.9/§16.123 [E013]</t>
+          <t>IRR tracker §16.122.9; DQ-6b Path A [E016][E024]</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Complete host sequence then freeze</t>
+          <t>Retain guarded split; no modernization by default</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>10/10 criteria met and freeze act effective; drift rule bound</t>
+          <t>Modernization accepted or continued interim state recorded</t>
         </is>
       </c>
     </row>
     <row r="18" ht="95" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>P-17</t>
+          <t>P-21</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -6497,27 +6497,27 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Row 45 — Release-readiness</t>
+          <t>Rows 30,32 — Governance</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Alias modernization / permanent pin architecture</t>
+          <t>PA-09 Gate 4 QE/H-12 pin designation</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>OPEN — NOT AUTHORIZED — OFF CRITICAL PATH</t>
+          <t>PA DECISION REQUIRED</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Only if PA commissions: B-1 governed IPD export or B-2 IRR broker-build redesign plus requalification tail; not an O-06 guard defect.</t>
+          <t>Choose C-1/C-2/C-3 and render exact Gate 4 QE/H-12 commit/tree/blobs/purpose; formal §4.5 scope conflict unresolved.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Separate PA act</t>
+          <t>PA decision; Limb A/native evidence if C-1</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -6532,320 +6532,320 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>IRR + IPD</t>
+          <t>IPD/IRR as scoped</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>CAP03-DQ6B-FOLLOW-ON-ALIAS-MODERNIZATION authority</t>
+          <t>G4-PIN act</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Interim guarded split is accepted; no current blocker</t>
+          <t>Gate 4 pin undesignated; §4.6 step 4 unsatisfied for L2c</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>PA act + scoped implementation + requalification evidence</t>
+          <t>Effective designation act + remote identities</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>IRR tracker §16.122.9; DQ-6b Path A [E016][E024]</t>
+          <t>IRR formal record §4.5; tracker §16.205.2 [E030][E031]</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Retain guarded split; no modernization by default</t>
+          <t>Render PA-09 choice</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Modernization accepted or continued interim state recorded</t>
+          <t>Exact Gate 4 pin designated; H-12 path unblocked</t>
         </is>
       </c>
     </row>
     <row r="19" ht="95" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>P-18</t>
+          <t>P-22</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>IRR implementation / deliverables</t>
+          <t>Qualification / admission gates</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Row 47 — Validation, Release-readiness</t>
+          <t>Rows 28,30,32 — Qualification</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Operator runbook figure restamp</t>
+          <t>Gate 4 S2/Limb A native run, H-12 L2c/S2a, S3, QE-1..11</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>PENDING — documentation drift</t>
+          <t>NOT STARTED / 0/11</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Restamp runbook headline figures to current head (108 files / 1377 tests) or add current-head verification pointer; start path already works.</t>
+          <t>Execute native S2/Limb A at designated pin; regenerate/adopt H-12; S3 preflight; QE-1..11 under adopted tiers; QE-8 uses RV-1 disposable-copy procedure.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>IRR documentation PR</t>
+          <t>PA-09 pin; P-1 provisioning; H-12 adoption</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>PA + operator</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>Operator</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Ordinary documentation admission</t>
+          <t>Gate 4 act execution grant; separate acceptance acts</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Runbook says 106/1350; current execution 108/1377</t>
+          <t>No designated final pin; P-1 unspent; H-12 not adopted at final pin</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Updated runbook + exact-head validation read-back</t>
+          <t>Native transcripts, H-12 adoption, S3/QE raw evidence, manifests</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>IRR docs/OPERATOR_RUNBOOK.md e94d2b80 [E006][E023]</t>
+          <t>IPD Gate 4 act; IRR PA-09/PA-10; RV-1 act [E012][E031][E034]</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Publish documentation-only restamp</t>
+          <t>Sequence after PA-09 and P-1; do not substitute Linux/CI for host QE</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Runbook figures reproduce at head or point to current verification baseline</t>
+          <t>S2/S2a/S3 complete; QE executed and recorded; acceptance still separate</t>
         </is>
       </c>
     </row>
     <row r="20" ht="95" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>P-19</t>
+          <t>P-23</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>IRR implementation / deliverables</t>
+          <t>Qualification / admission gates</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Row 48 — Governance</t>
+          <t>Rows 28,30,32 — Acceptance</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Tracker allocation conflict with open PR #398</t>
+          <t>Gate C acceptance for QE-11 subset</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>OPEN — coordination required</t>
+          <t>NOT RENDERED</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Preserve PR #398 proposed §16.230/CV-CORR-210/V1806-V1817; this reassessment allocates §16.231/CV-CORR-211 to avoid collision if both merge.</t>
+          <t>Render separate Gate C result-acceptance act for Q1-Q4/Q9-Q11 after subset execution.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>PR #398 merge/close outcome</t>
+          <t>QE-11 subset execution</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>Gate C acceptance authority</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>Operator + PA</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Identifier allocation convention</t>
+          <t>Separate Gate C acceptance act</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Open PR proposes next main allocation</t>
+          <t>Execution grant is not acceptance</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>No duplicate consumed identifiers after merge/rebase</t>
+          <t>Accepted Gate C subset result + raw evidence</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>IRR PR #398; tracker §16.229 next-free [E004][E010]</t>
+          <t>IPD Gate 4 act §7 [E012]</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Reconcile with main before merge; do not reuse PR #398 identifiers</t>
+          <t>Execute subset then seek acceptance</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Allocations unique on final main; historical records preserved</t>
+          <t>QE-11 'passed and accepted' limb satisfied by separate act</t>
         </is>
       </c>
     </row>
     <row r="21" ht="95" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>P-20</t>
+          <t>P-24</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>IPD implementation / deliverables</t>
+          <t>Qualification / admission gates</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Row 48 — Evidence, Governance</t>
+          <t>Rows 28,30,32 — Acceptance</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>IPD tracker stale P-1 footer</t>
+          <t>Gate 4 result acceptance / U4</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>PENDING — documentation conflict</t>
+          <t>NOT RENDERED</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Correct IPD tracker footer 'P-1 NOT AUTHORIZED' by dated pointer to IRR P1-F effective authorization; do not rewrite IRR authority from IPD.</t>
+          <t>Render Gate 4 result acceptance after QE evidence integrity and Gate C subset acceptance.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>IPD documentation PR</t>
+          <t>QE + Gate C acceptance</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>IPD</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>IPD</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>IPD</t>
+          <t>Operator + PA</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>IPD ordinary documentation admission; IRR owns P1-F</t>
+          <t>U4 acceptance act</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>IPD footer conflicts with IRR main §16.206/§16.229</t>
+          <t>QE 0/11; no acceptance</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>IPD dated pointer + remote read-back</t>
+          <t>Effective U4 act + evidence read-back</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>IPD tracker 31fd3b84; IRR P1-F act [E005][E011]</t>
+          <t>IPD Gate 4 act §6 S6; IPD tracker U4 [E012][E035]</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>Publish IPD-side pointer only</t>
+          <t>Complete qualification then acceptance</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>IPD tracker no longer asserts stale current P-1 authority; IRR act unchanged</t>
+          <t>Gate 4 accepted for named scope; not inferred from tests</t>
         </is>
       </c>
     </row>
     <row r="22" ht="95" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>P-21</t>
+          <t>P-25</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>PA decisions / governance</t>
+          <t>Qualification / admission gates</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,32 — Governance</t>
+          <t>Rows 28,30,32 — Release-readiness</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>PA-09 Gate 4 QE/H-12 pin designation</t>
+          <t>Gate 5 / CV-52 / U5 admission</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>PA DECISION REQUIRED</t>
+          <t>NOT INITIATED / NOT ADMITTED</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Choose C-1/C-2/C-3 and render exact Gate 4 QE/H-12 commit/tree/blobs/purpose; formal §4.5 scope conflict unresolved.</t>
+          <t>Render Gate 5 admission after Gate 4 acceptance and DQ-4 freeze; name qualified commits and lifted fences only.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>PA decision; Limb A/native evidence if C-1</t>
+          <t>U4 + DQ-4 + DR-4r/DQ-3 boundary</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -6860,44 +6860,44 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>IPD/IRR as scoped</t>
+          <t>IRR + IPD</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>G4-PIN act</t>
+          <t>U5 admission act</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Gate 4 pin undesignated; §4.6 step 4 unsatisfied for L2c</t>
+          <t>CV-52 blocked; durable reads not granted</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Effective designation act + remote identities</t>
+          <t>Effective admission act + named commits + fence disposition</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>IRR formal record §4.5; tracker §16.205.2 [E030][E031]</t>
+          <t>IRR tracker CV-52; IPD tracker U5 [E004][E035]</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Render PA-09 choice</t>
+          <t>Progress upstream gates; no admission by CI</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Exact Gate 4 pin designated; H-12 path unblocked</t>
+          <t>Gate 5 admitted for exact scope or recorded no</t>
         </is>
       </c>
     </row>
     <row r="23" ht="95" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>P-22</t>
+          <t>P-26</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -6907,32 +6907,32 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Rows 28,30,32 — Qualification</t>
+          <t>Rows 28,30 — Release-readiness</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Gate 4 S2/Limb A native run, H-12 L2c/S2a, S3, QE-1..11</t>
+          <t>U6 operational write authorization / durable:true / 503 lift</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>NOT STARTED / 0/11</t>
+          <t>NOT AUTHORIZED</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Execute native S2/Limb A at designated pin; regenerate/adopt H-12; S3 preflight; QE-1..11 under adopted tiers; QE-8 uses RV-1 disposable-copy procedure.</t>
+          <t>Render separate U6 act satisfying W-1 after Gate 5; no code/CI result can supply it.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>PA-09 pin; P-1 provisioning; H-12 adoption</t>
+          <t>Gate 5 admission</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>PA + operator</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -6942,79 +6942,79 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Operator</t>
+          <t>IPD + IRR</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Gate 4 act execution grant; separate acceptance acts</t>
+          <t>U6 write authorization act</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>No designated final pin; P-1 unspent; H-12 not adopted at final pin</t>
+          <t>evaluatePortSaveGuard hard-false; W-1(3)/W-1(4) unmet</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Native transcripts, H-12 adoption, S3/QE raw evidence, manifests</t>
+          <t>Effective U6 act + qualified write evidence + guard change authority</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>IPD Gate 4 act; IRR PA-09/PA-10; RV-1 act [E012][E031][E034]</t>
+          <t>IPD tracker U6; IPD portfolio_store guard [E014][E035]</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Sequence after PA-09 and P-1; do not substitute Linux/CI for host QE</t>
+          <t>Keep writes refused until U6</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>S2/S2a/S3 complete; QE executed and recorded; acceptance still separate</t>
+          <t>Operational writes authorized only by effective act and qualified evidence</t>
         </is>
       </c>
     </row>
     <row r="24" ht="95" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>P-23</t>
+          <t>P-27</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Qualification / admission gates</t>
+          <t>PA decisions / governance</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Rows 28,30,32 — Acceptance</t>
+          <t>Rows 30,32 — Governance</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Gate C acceptance for QE-11 subset</t>
+          <t>PA-01 source-authority conflict</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>NOT RENDERED</t>
+          <t>PARTLY RESOLVED — documentary conflict remains</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Render separate Gate C result-acceptance act for Q1-Q4/Q9-Q11 after subset execution.</t>
+          <t>Render source-confirmation/disposition for designation-record vs rulings-record conflict; A-Q4→PA-02, G4P-1→PA-09.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>QE-11 subset execution</t>
+          <t>PA decision</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Gate C acceptance authority</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -7024,74 +7024,74 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Operator + PA</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Separate Gate C acceptance act</t>
+          <t>PA-01 act</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Execution grant is not acceptance</t>
+          <t>Record conflict not resolved by assumption</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Accepted Gate C subset result + raw evidence</t>
+          <t>Effective source-confirmation act</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>IPD Gate 4 act §7 [E012]</t>
+          <t>IRR tracker §16.205.2; PA package PA-01 [E004][E030]</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Execute subset then seek acceptance</t>
+          <t>Put narrow source confirmation to PA</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>QE-11 'passed and accepted' limb satisfied by separate act</t>
+          <t>Conflict expressly resolved or retained; no execution dependency inferred</t>
         </is>
       </c>
     </row>
     <row r="25" ht="95" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>P-24</t>
+          <t>P-28</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Qualification / admission gates</t>
+          <t>PA decisions / governance</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Rows 28,30,32 — Acceptance</t>
+          <t>Rows 30,32 — Governance</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Gate 4 result acceptance / U4</t>
+          <t>PA-02 A-Q4 / PR #96 paths</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>NOT RENDERED</t>
+          <t>PA DECISION REQUIRED — documentary</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Render Gate 4 result acceptance after QE evidence integrity and Gate C subset acceptance.</t>
+          <t>Decide whether 521d5482 blob is the authorizing record for the two PR #96 paths; it names paths but disclaims grant.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>QE + Gate C acceptance</t>
+          <t>PA decision</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -7106,74 +7106,74 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Operator + PA</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>U4 acceptance act</t>
+          <t>A-Q4 determination</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>QE 0/11; no acceptance</t>
+          <t>No PA ruling; PA-01 not a genuine prerequisite</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Effective U4 act + evidence read-back</t>
+          <t>Effective A-Q4 act</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>IPD Gate 4 act §6 S6; IPD tracker U4 [E012][E035]</t>
+          <t>IRR disposition blob 521d5482; IPD AQ5 correction [E030][E032]</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Complete qualification then acceptance</t>
+          <t>Render A-Q4 decision</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>Gate 4 accepted for named scope; not inferred from tests</t>
+          <t>Authorizing record question answered; no gate inferred</t>
         </is>
       </c>
     </row>
     <row r="26" ht="95" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>P-25</t>
+          <t>P-29</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Qualification / admission gates</t>
+          <t>PA decisions / governance</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Rows 28,30,32 — Release-readiness</t>
+          <t>Rows 30,32 — Governance</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Gate 5 / CV-52 / U5 admission</t>
+          <t>PA-03 A-Q5 sequencing ratification</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>NOT INITIATED / NOT ADMITTED</t>
+          <t>EFFECTS RESOLVED — express ratification open</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Render Gate 5 admission after Gate 4 acceptance and DQ-4 freeze; name qualified commits and lifted fences only.</t>
+          <t>Ratify sequencing deviation / mechanism attribution; executed blob designations stand on A-Q1/A-Q2.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>U4 + DQ-4 + DR-4r/DQ-3 boundary</t>
+          <t>PA decision</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -7188,74 +7188,74 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>IRR + IPD</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>U5 admission act</t>
+          <t>PA-03 ratification</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>CV-52 blocked; durable reads not granted</t>
+          <t>IPD correction marks mechanism attribution PA-reserved</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Effective admission act + named commits + fence disposition</t>
+          <t>Effective ratification/source-confirmation statement</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>IRR tracker CV-52; IPD tracker U5 [E004][E035]</t>
+          <t>IPD AQ5 act correction; IRR rulings §8 [E032]</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>Progress upstream gates; no admission by CI</t>
+          <t>Render narrow ratification</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>Gate 5 admitted for exact scope or recorded no</t>
+          <t>Sequencing attribution resolved; no re-execution of blob amendment</t>
         </is>
       </c>
     </row>
     <row r="27" ht="95" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>P-26</t>
+          <t>P-30</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Qualification / admission gates</t>
+          <t>PA decisions / governance</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Rows 28,30 — Release-readiness</t>
+          <t>Rows 25,41 — Governance</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>U6 operational write authorization / durable:true / 503 lift</t>
+          <t>PA-17 REG-12 Company Identity Authority mapping</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>NOT AUTHORIZED</t>
+          <t>NO DISPOSITION — owner decision</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Render separate U6 act satisfying W-1 after Gate 5; no code/CI result can supply it.</t>
+          <t>Designate or decline Company Identity Authority naming bounded domain/source/consumer; not a P-1/Gate 4 prerequisite.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Gate 5 admission</t>
+          <t>PA decision</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -7270,156 +7270,156 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>IPD + IRR</t>
+          <t>IRR + IPD</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>U6 write authorization act</t>
+          <t>REG-12 mapping act</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>evaluatePortSaveGuard hard-false; W-1(3)/W-1(4) unmet</t>
+          <t>No CIA designated; mapping blocker unresolved</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Effective U6 act + qualified write evidence + guard change authority</t>
+          <t>Effective designation/declination act</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>IPD tracker U6; IPD portfolio_store guard [E014][E035]</t>
+          <t>IRR tracker §16.198/§16.205.2; CV-43/D115 [E004][E030]</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Keep writes refused until U6</t>
+          <t>Put REG-12 mapping decision to PA</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>Operational writes authorized only by effective act and qualified evidence</t>
+          <t>Mapping blocker resolved or expressly declined</t>
         </is>
       </c>
     </row>
     <row r="28" ht="95" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>P-27</t>
+          <t>P-31</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>PA decisions / governance</t>
+          <t>Evidence / certification / verification</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,32 — Governance</t>
+          <t>Rows 30,34 — Validation</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>PA-01 source-authority conflict</t>
+          <t>V1295 endpoint literal test binding</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>PARTLY RESOLVED — documentary conflict remains</t>
+          <t>NOT MET</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Render source-confirmation/disposition for designation-record vs rulings-record conflict; A-Q4→PA-02, G4P-1→PA-09.</t>
+          <t>Bind designated endpoint literal \\.\pipe\iips-user-portfolio-v1 in an authorized test, or record PA disposition.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>PA decision</t>
+          <t>Authorized test/evidence act</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>IRR/IPD test owner</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>IRR + IPD</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>PA-01 act</t>
+          <t>PA disposition if not tested</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Record conflict not resolved by assumption</t>
+          <t>No test binds the literal; F-S2-3</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Effective source-confirmation act</t>
+          <t>Test evidence or PA disposition</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>IRR tracker §16.205.2; PA package PA-01 [E004][E030]</t>
+          <t>IRR tracker V1295 [E004]</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>Put narrow source confirmation to PA</t>
+          <t>Add binding under existing test authority if available; otherwise PA disposition</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Conflict expressly resolved or retained; no execution dependency inferred</t>
+          <t>V1295 met or expressly disposed</t>
         </is>
       </c>
     </row>
     <row r="29" ht="95" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>P-28</t>
+          <t>P-32</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>PA decisions / governance</t>
+          <t>Cross-repository integration / dependencies</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,32 — Governance</t>
+          <t>Rows 28,30,31 — Integration</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>PA-02 A-Q4 / PR #96 paths</t>
+          <t>DR-2 / DR-4r-DQ-3 operational closure</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>PA DECISION REQUIRED — documentary</t>
+          <t>IMPLEMENTATION COMPLETE — operational closure open</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Decide whether 521d5482 blob is the authorizing record for the two PR #96 paths; it names paths but disclaims grant.</t>
+          <t>Close cross-repo operational line only after DQ-4 freeze and Gate 5; do not reopen provider/consumer implementation.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>PA decision</t>
+          <t>DQ-4 + Gate 5</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -7429,89 +7429,89 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>IRR + IPD</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>IRR + IPD</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>A-Q4 determination</t>
+          <t>Downstream admission acts</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>No PA ruling; PA-01 not a genuine prerequisite</t>
+          <t>Implementation merged; operational closure not established</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Effective A-Q4 act</t>
+          <t>Closure record referencing freeze/admission</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>IRR disposition blob 521d5482; IPD AQ5 correction [E030][E032]</t>
+          <t>IRR §§16.117-16.118; IPD DR-2 verification [E004][E005]</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Render A-Q4 decision</t>
+          <t>Track as downstream closure, not new implementation</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Authorizing record question answered; no gate inferred</t>
+          <t>Operational closure recorded after gates; no duplicate code work</t>
         </is>
       </c>
     </row>
     <row r="30" ht="95" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>P-29</t>
+          <t>P-33</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>PA decisions / governance</t>
+          <t>IRR implementation / deliverables</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,32 — Governance</t>
+          <t>Rows 30,48 — Governance</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>PA-03 A-Q5 sequencing ratification</t>
+          <t>G14 final cross-stage reconciliation</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>EFFECTS RESOLVED — express ratification open</t>
+          <t>BLOCKED — dependency assessment published; final G14 NOT STARTED</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Ratify sequencing deviation / mechanism attribution; executed blob designations stand on A-Q1/A-Q2.</t>
+          <t>Perform final IRR cross-stage reconciliation only after G2-G13 close. Current assessment identifies incomplete PA decisions, P-1 consumption reconciliation/execution, S3, QE, DQ-4, Gate 4 acceptance and Gate 5 admission.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>PA decision</t>
+          <t>G2-G13 completion</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>PA + Operator + IRR + IPD</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -7521,156 +7521,156 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>PA-03 ratification</t>
+          <t>Existing one-pass authorization; no upstream gate may be inferred closed</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>IPD correction marks mechanism attribution PA-reserved</t>
+          <t>G6 P-1 consumption NOT RECONCILED; G7 S3 not started; G8 QE 0/11; G9 DQ-4 8/10; G10 Gate 4 acceptance not rendered; G11 Gate 5 not initiated</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Effective ratification/source-confirmation statement</t>
+          <t>Final G14 register + tracker pointer after upstream closure</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>IPD AQ5 act correction; IRR rulings §8 [E032]</t>
+          <t>IRR docs/integration/IIPS_v3.0_CAP03_G14_DEPENDENCY_ASSESSMENT_2026-10-31.md; IRR tracker §16.233; IPD main@527f811 [E040][E041]</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>Render narrow ratification</t>
+          <t>Progress upstream PA/operator gates; do not declare G14 complete</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Sequencing attribution resolved; no re-execution of blob amendment</t>
+          <t>All G2-G13 statuses reconciled from evidence and final G14 record published</t>
         </is>
       </c>
     </row>
     <row r="31" ht="95" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>P-30</t>
+          <t>P-34</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>PA decisions / governance</t>
+          <t>External / infrastructure blockers</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Rows 25,41 — Governance</t>
+          <t>Rows 19,27,30 — E2E</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>PA-17 REG-12 Company Identity Authority mapping</t>
+          <t>Designated Windows host / operator availability</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>NO DISPOSITION — owner decision</t>
+          <t>EXTERNAL — required for host-only evidence</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Designate or decline Company Identity Authority naming bounded domain/source/consumer; not a P-1/Gate 4 prerequisite.</t>
+          <t>Provide designated Windows host/operator for P-1, S3/QE, O-09 and macro browser evidence; waivers remove governance blockers but not runtime facts.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>PA decision</t>
+          <t>Operator host access</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>IRR + IPD</t>
+          <t>Operator</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>REG-12 mapping act</t>
+          <t>Existing PA host profile / waivers</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>No CIA designated; mapping blocker unresolved</t>
+          <t>Arena has no Windows host; host facts unverified</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Effective designation/declination act</t>
+          <t>Host transcripts and run records</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>IRR tracker §16.198/§16.205.2; CV-43/D115 [E004][E030]</t>
+          <t>IRR PA host profile; tracker §16.229 [E004][E011]</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>Put REG-12 mapping decision to PA</t>
+          <t>Schedule operator host sessions</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>Mapping blocker resolved or expressly declined</t>
+          <t>Required host evidence captured; no waiver converted to PASS</t>
         </is>
       </c>
     </row>
     <row r="32" ht="95" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>P-31</t>
+          <t>P-35</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Evidence / certification / verification</t>
+          <t>External / infrastructure blockers</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,34 — Validation</t>
+          <t>Row 19 — Wiring, E2E</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>V1295 endpoint literal test binding</t>
+          <t>MoSPI egress for current-environment macro capture</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>NOT MET</t>
+          <t>EXTERNAL — sandbox no-egress</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Bind designated endpoint literal \\.\pipe\iips-user-portfolio-v1 in an authorized test, or record PA disposition.</t>
+          <t>Provide operator network egress if current-environment live macro capture is required; operator Windows live E2E already established.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Authorized test/evidence act</t>
+          <t>Network egress</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>IRR/IPD test owner</t>
+          <t>Operator</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -7680,131 +7680,131 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>IRR + IPD</t>
+          <t>Operator</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>PA disposition if not tested</t>
+          <t>None for existing operator evidence</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>No test binds the literal; F-S2-3</t>
+          <t>Sandbox fetch failed after 4 attempts</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Test evidence or PA disposition</t>
+          <t>Live capture transcript from egress-capable host</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>IRR tracker V1295 [E004]</t>
+          <t>IRR probe 502; tracker §16.31 [E008][E027]</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>Add binding under existing test authority if available; otherwise PA disposition</t>
+          <t>Use operator evidence or capture with egress</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>V1295 met or expressly disposed</t>
+          <t>Current-environment live capture evidenced or residual retained</t>
         </is>
       </c>
     </row>
     <row r="33" ht="95" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>P-32</t>
+          <t>P-36</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Cross-repository integration / dependencies</t>
+          <t>Evidence / certification / verification</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Rows 28,30,31 — Integration</t>
+          <t>Rows 30,45 — Evidence, Validation</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>DR-2 / DR-4r-DQ-3 operational closure</t>
+          <t>Historical S2 emitted bytes / S04-compatible retained bundle</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>IMPLEMENTATION COMPLETE — operational closure open</t>
+          <t>PARTIAL — release assets byte-verified; S04 bundle acceptance pending</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Close cross-repo operational line only after DQ-4 freeze and Gate 5; do not reopen provider/consumer implementation.</t>
+          <t>PR #398 verified the four recovery-release assets and all 1,140 ZIP payload hashes against the original inventory. The four-asset release is not the S04 sealed-directory bundle; obtain/accept the complete sealed bundle or retain the limitation.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>DQ-4 + Gate 5</t>
+          <t>S04-compatible sealed bundle / PA disposition</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>Operator + IRR</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>IRR + IPD</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>IRR + IPD</t>
+          <t>Operator + IRR</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Downstream admission acts</t>
+          <t>No rebuild/fabrication; S04 contract must not be weakened</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Implementation merged; operational closure not established</t>
+          <t>Release layout lacks canonical MANIFEST/SHA256SUMS/seal/reports/dist bundle required by S04</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Closure record referencing freeze/admission</t>
+          <t>S04 bundle read-back + per-entry hash match, or dated limitation/disposition</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>IRR §§16.117-16.118; IPD DR-2 verification [E004][E005]</t>
+          <t>IRR PR #398 §16.232; recovery release cap03-s2-recovery-20261031-212225 [E010][E037]</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>Track as downstream closure, not new implementation</t>
+          <t>Assemble/verify the canonical sealed bundle from exact original bytes if available; otherwise retain limitation</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>Operational closure recorded after gates; no duplicate code work</t>
+          <t>S04-compatible retention accepted or limitation formally retained; no S2/P-1 authority inferred</t>
         </is>
       </c>
     </row>
     <row r="34" ht="95" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>P-33</t>
+          <t>P-37</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>IRR implementation / deliverables</t>
+          <t>PA decisions / governance</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -7814,109 +7814,109 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>G14 final cross-stage reconciliation</t>
+          <t>P1-F consumption-state reconciliation</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>NOT DONE</t>
+          <t>UNRECONCILED in open PR #398; authoritative main records UNSPENT</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Perform final IRR cross-stage reconciliation after upstream groups/gates complete.</t>
+          <t>Reconcile operator-reported S00/S04 stops from raw host evidence and render/record the authoritative consumption state; do not infer consumed/unspent from launcher completion.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>G2-G13 completion</t>
+          <t>Raw host run records + PA/authority reconciliation</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>Operator + IRR</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Existing one-pass authorization</t>
+          <t>PA/authority record; no retry authority</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Upstream gates incomplete</t>
+          <t>PR #398 proposes S00-P1F-CONSUMPTION-RECONCILED fail-closed; not merged</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Final reconciliation record + tracker pointer</t>
+          <t>Raw evidence + authoritative tracker/act reconciliation</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>IPD tracker G14; IRR tracker [E004][E005]</t>
+          <t>IRR tracker §16.229; PR #398 [E004][E010]</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>Wait for upstream closure; then reconcile</t>
+          <t>Collect raw host evidence; reconcile before any further Execute boundary</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>All upstream statuses reconciled without inferred closure</t>
+          <t>Consumption state expressly reconciled; one-attempt guard preserved</t>
         </is>
       </c>
     </row>
     <row r="35" ht="95" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>P-34</t>
+          <t>P-38</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>External / infrastructure blockers</t>
+          <t>PA decisions / governance</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Rows 19,27,30 — E2E</t>
+          <t>Rows 30,32 — Governance</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Designated Windows host / operator availability</t>
+          <t>PA-05 B-Q6 aa43dec2 eligibility</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>EXTERNAL — required for host-only evidence</t>
+          <t>OPTIONAL — no operation depends</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Provide designated Windows host/operator for P-1, S3/QE, O-09 and macro browser evidence; waivers remove governance blockers but not runtime facts.</t>
+          <t>PA may decide whether IPD aa43dec2 is eligible as a Matter B designation target; no current P-1/S2/Gate 4 step depends on it.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Operator host access</t>
+          <t>PA decision</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Operator</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -7926,208 +7926,208 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Operator</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Existing PA host profile / waivers</t>
+          <t>PA-05 optional act</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Arena has no Windows host; host facts unverified</t>
+          <t>No operation depends; recommendation not adopted</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Host transcripts and run records</t>
+          <t>Effective eligibility disposition if pursued</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>IRR PA host profile; tracker §16.229 [E004][E011]</t>
+          <t>IRR PA package PA-05 [E030]</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>Schedule operator host sessions</t>
+          <t>No action required unless PA pursues</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>Required host evidence captured; no waiver converted to PASS</t>
+          <t>Optional decision rendered or retained as non-blocking</t>
         </is>
       </c>
     </row>
     <row r="36" ht="95" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>P-35</t>
+          <t>P-39</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>External / infrastructure blockers</t>
+          <t>PA decisions / governance</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Row 19 — Wiring, E2E</t>
+          <t>Rows 30,32,48 — Governance</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>MoSPI egress for current-environment macro capture</t>
+          <t>PA-07 label scheme</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>EXTERNAL — sandbox no-egress</t>
+          <t>OPTIONAL — label-only</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Provide operator network egress if current-environment live macro capture is required; operator Windows live E2E already established.</t>
+          <t>PA may adopt label scheme for S2 uses/matter aliases/collisions; no gate or operation depends on labels.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Network egress</t>
+          <t>PA decision</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Operator</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Operator</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>None for existing operator evidence</t>
+          <t>PA-07 optional act</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Sandbox fetch failed after 4 attempts</t>
+          <t>Label-only; no substantive blocker</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Live capture transcript from egress-capable host</t>
+          <t>Effective label disposition if pursued</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>IRR probe 502; tracker §16.31 [E008][E027]</t>
+          <t>IRR PA package PA-07 [E030]</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>Use operator evidence or capture with egress</t>
+          <t>No action required unless PA pursues</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>Current-environment live capture evidenced or residual retained</t>
+          <t>Labels adopted or retained descriptive; no inferred blocker</t>
         </is>
       </c>
     </row>
     <row r="37" ht="95" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>P-36</t>
+          <t>P-40</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Evidence / certification / verification</t>
+          <t>PA decisions / governance</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,45 — Evidence, Validation</t>
+          <t>Rows 30,32 — Governance</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Historical S2 emitted bytes / dist-artifacts.zip retention</t>
+          <t>PA-11 successor D-INST instrument adoption</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>PENDING — historical bytes unavailable</t>
+          <t>CONDITIONAL — untriggered</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Obtain and independently hash the exact original emitted S2 bytes/archive, or retain the limitation; PR #398 adds future capture/retention but does not verify historical bytes.</t>
+          <t>If a successor D-2 instrument is to be used, adopt its identity and satisfy T-1 parse/run validation before first use; current v2 identity unchanged.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Original host emitted bytes / archive</t>
+          <t>PA adoption + T-1 before first use</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Operator</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Operator + IRR</t>
+          <t>IRR + Operator</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>No rebuild/fabrication; PA disposition if historical verification is waived</t>
+          <t>PA-11 act; PA-12/A6 route as applicable</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Preserved admitted S2 folder has inventories but no dist-artifacts.zip/emitted files</t>
+          <t>No successor adoption record; trigger absent</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Original archive read-back + per-entry hash match, or dated limitation/disposition</t>
+          <t>Adoption act + validation evidence before use</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>IRR PR #398; S2 admitted evidence [E010][E033]</t>
+          <t>IRR PA package PA-11; rulings D-Q/PF10 [E030]</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>Do not rebuild historical evidence; capture future runs under corrected instrument</t>
+          <t>Do not use successor instrument without adoption</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>Historical bytes verified or limitation formally retained; future retention gate effective</t>
+          <t>Successor adopted and validated, or path remains untriggered</t>
         </is>
       </c>
     </row>
     <row r="38" ht="95" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>P-37</t>
+          <t>P-41</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -8137,27 +8137,27 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,48 — Governance</t>
+          <t>Row 35 — Governance</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>P1-F consumption-state reconciliation</t>
+          <t>PA-16 REG-11 formal closure/reopen</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>UNRECONCILED in open PR #398; authoritative main records UNSPENT</t>
+          <t>OPTIONAL — Option C deferral retained</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Reconcile operator-reported S00/S04 stops from raw host evidence and render/record the authoritative consumption state; do not infer consumed/unspent from launcher completion.</t>
+          <t>PA may retain Option C, formally close, or reopen REG-11; no downstream step depends on it.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Raw host run records + PA/authority reconciliation</t>
+          <t>PA decision</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -8172,44 +8172,44 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Operator + IRR</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>PA/authority record; no retry authority</t>
+          <t>PA-16 optional act</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>PR #398 proposes S00-P1F-CONSUMPTION-RECONCILED fail-closed; not merged</t>
+          <t>REG-11 not closed; no dependent operation</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>Raw evidence + authoritative tracker/act reconciliation</t>
+          <t>Effective REG-11 disposition if pursued</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>IRR tracker §16.229; PR #398 [E004][E010]</t>
+          <t>IRR PA package PA-16; tracker §16.112/§16.199 [E030]</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>Collect raw host evidence; reconcile before any further Execute boundary</t>
+          <t>No action required unless PA pursues</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>Consumption state expressly reconciled; one-attempt guard preserved</t>
+          <t>REG-11 disposition rendered or deferral retained</t>
         </is>
       </c>
     </row>
     <row r="39" ht="95" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>P-38</t>
+          <t>P-42</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -8224,17 +8224,17 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>PA-05 B-Q6 aa43dec2 eligibility</t>
+          <t>PA-18 L2b action requirement</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>OPTIONAL — no operation depends</t>
+          <t>NO TRIGGER FOUND</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>PA may decide whether IPD aa43dec2 is eligible as a Matter B designation target; no current P-1/S2/Gate 4 step depends on it.</t>
+          <t>PA may decide whether any L2b action is required; P1-F list does not include L2b and no operation requires it.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -8259,22 +8259,22 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>PA-05 optional act</t>
+          <t>PA-18 optional act</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>No operation depends; recommendation not adopted</t>
+          <t>No trigger; non-blocking</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>Effective eligibility disposition if pursued</t>
+          <t>Effective no-action/action decision if pursued</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>IRR PA package PA-05 [E030]</t>
+          <t>IRR PA package PA-18; tracker §16.122.9 [E030]</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
@@ -8284,44 +8284,44 @@
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>Optional decision rendered or retained as non-blocking</t>
+          <t>L2b requirement expressly decided or remains untriggered</t>
         </is>
       </c>
     </row>
     <row r="40" ht="95" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>P-39</t>
+          <t>P-43</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>PA decisions / governance</t>
+          <t>Cross-repository integration / dependencies</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,32,48 — Governance</t>
+          <t>Rows 30,32 — Integration, Qualification</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>PA-07 label scheme</t>
+          <t>CV-20 user-portfolio authority sequencing</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>OPTIONAL — label-only</t>
+          <t>ACTIVE — qualification/admission sequence</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>PA may adopt label scheme for S2 uses/matter aliases/collisions; no gate or operation depends on labels.</t>
+          <t>Carry the accepted G-2 architecture through Gate 4 qualification, formal acceptance and separate admission; architecture itself is not open.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>PA decision</t>
+          <t>Gate 4 / Gate 5 sequence</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -8336,74 +8336,74 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>IRR + IPD + Operator</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>PA-07 optional act</t>
+          <t>Separate qualification/acceptance/admission acts</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Label-only; no substantive blocker</t>
+          <t>Durable implementation unadmitted; live seam fenced</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>Effective label disposition if pursued</t>
+          <t>Qualified commits + acceptance + admission act</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>IRR PA package PA-07 [E030]</t>
+          <t>IRR tracker CV-20; G-2 decision [E004]</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>No action required unless PA pursues</t>
+          <t>Progress P-09..P-26 chain; no re-architecture</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>Labels adopted or retained descriptive; no inferred blocker</t>
+          <t>CV-20 closed by qualified admission or recorded disposition</t>
         </is>
       </c>
     </row>
     <row r="41" ht="95" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>P-40</t>
+          <t>P-44</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>PA decisions / governance</t>
+          <t>Cross-repository integration / dependencies</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Rows 30,32 — Governance</t>
+          <t>Row 28 — Integration, Acceptance</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>PA-11 successor D-INST instrument adoption</t>
+          <t>CV-39 broker ingestion into G-2 admission</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>CONDITIONAL — untriggered</t>
+          <t>DEFERRED — bounded Gate 3 accepted</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>If a successor D-2 instrument is to be used, adopt its identity and satisfy T-1 parse/run validation before first use; current v2 identity unchanged.</t>
+          <t>Carry broker ingestion into Gate 4/Gate 5 admission with durability, UNRESOLVED preservation, idempotent re-import and restart/read evidence; no independent runtime enablement.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>PA adoption + T-1 before first use</t>
+          <t>CV-20 Gate 4/Gate 5 sequence</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -8418,370 +8418,42 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>IRR + Operator</t>
+          <t>IPD + IRR + Operator</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>PA-11 act; PA-12/A6 route as applicable</t>
+          <t>Gate 4/Gate 5 acts</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>No successor adoption record; trigger absent</t>
+          <t>Bounded implementation accepted; operational admission deferred</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>Adoption act + validation evidence before use</t>
+          <t>Import→persist→restart→read evidence + admission act</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>IRR PA package PA-11; rulings D-Q/PF10 [E030]</t>
+          <t>IRR tracker CV-39; IPD Gate 3 acceptance [E004][E035]</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Do not use successor instrument without adoption</t>
+          <t>Sequence with P-22..P-26; no separate enablement</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>Successor adopted and validated, or path remains untriggered</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="95" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>P-41</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>PA decisions / governance</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Row 35 — Governance</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>PA-16 REG-11 formal closure/reopen</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>OPTIONAL — Option C deferral retained</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>PA may retain Option C, formally close, or reopen REG-11; no downstream step depends on it.</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>PA decision</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>IRR</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>PA-16 optional act</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>REG-11 not closed; no dependent operation</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>Effective REG-11 disposition if pursued</t>
-        </is>
-      </c>
-      <c r="N42" s="2" t="inlineStr">
-        <is>
-          <t>IRR PA package PA-16; tracker §16.112/§16.199 [E030]</t>
-        </is>
-      </c>
-      <c r="O42" s="2" t="inlineStr">
-        <is>
-          <t>No action required unless PA pursues</t>
-        </is>
-      </c>
-      <c r="P42" s="2" t="inlineStr">
-        <is>
-          <t>REG-11 disposition rendered or deferral retained</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="95" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>P-42</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>PA decisions / governance</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Rows 30,32 — Governance</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>PA-18 L2b action requirement</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>NO TRIGGER FOUND</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>PA may decide whether any L2b action is required; P1-F list does not include L2b and no operation requires it.</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>PA decision</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>IRR</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>PA-18 optional act</t>
-        </is>
-      </c>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>No trigger; non-blocking</t>
-        </is>
-      </c>
-      <c r="M43" s="2" t="inlineStr">
-        <is>
-          <t>Effective no-action/action decision if pursued</t>
-        </is>
-      </c>
-      <c r="N43" s="2" t="inlineStr">
-        <is>
-          <t>IRR PA package PA-18; tracker §16.122.9 [E030]</t>
-        </is>
-      </c>
-      <c r="O43" s="2" t="inlineStr">
-        <is>
-          <t>No action required unless PA pursues</t>
-        </is>
-      </c>
-      <c r="P43" s="2" t="inlineStr">
-        <is>
-          <t>L2b requirement expressly decided or remains untriggered</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="95" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>P-43</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Cross-repository integration / dependencies</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Rows 30,32 — Integration, Qualification</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>CV-20 user-portfolio authority sequencing</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE — qualification/admission sequence</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Carry the accepted G-2 architecture through Gate 4 qualification, formal acceptance and separate admission; architecture itself is not open.</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>Gate 4 / Gate 5 sequence</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>IRR + IPD + Operator</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr">
-        <is>
-          <t>Separate qualification/acceptance/admission acts</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>Durable implementation unadmitted; live seam fenced</t>
-        </is>
-      </c>
-      <c r="M44" s="2" t="inlineStr">
-        <is>
-          <t>Qualified commits + acceptance + admission act</t>
-        </is>
-      </c>
-      <c r="N44" s="2" t="inlineStr">
-        <is>
-          <t>IRR tracker CV-20; G-2 decision [E004]</t>
-        </is>
-      </c>
-      <c r="O44" s="2" t="inlineStr">
-        <is>
-          <t>Progress P-09..P-26 chain; no re-architecture</t>
-        </is>
-      </c>
-      <c r="P44" s="2" t="inlineStr">
-        <is>
-          <t>CV-20 closed by qualified admission or recorded disposition</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="95" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>P-44</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Cross-repository integration / dependencies</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Row 28 — Integration, Acceptance</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>CV-39 broker ingestion into G-2 admission</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>DEFERRED — bounded Gate 3 accepted</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>Carry broker ingestion into Gate 4/Gate 5 admission with durability, UNRESOLVED preservation, idempotent re-import and restart/read evidence; no independent runtime enablement.</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>CV-20 Gate 4/Gate 5 sequence</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>IPD + IRR + Operator</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>Gate 4/Gate 5 acts</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>Bounded implementation accepted; operational admission deferred</t>
-        </is>
-      </c>
-      <c r="M45" s="2" t="inlineStr">
-        <is>
-          <t>Import→persist→restart→read evidence + admission act</t>
-        </is>
-      </c>
-      <c r="N45" s="2" t="inlineStr">
-        <is>
-          <t>IRR tracker CV-39; IPD Gate 3 acceptance [E004][E035]</t>
-        </is>
-      </c>
-      <c r="O45" s="2" t="inlineStr">
-        <is>
-          <t>Sequence with P-22..P-26; no separate enablement</t>
-        </is>
-      </c>
-      <c r="P45" s="2" t="inlineStr">
-        <is>
           <t>Durable import admitted only as part of G-2 admission</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P45"/>
+  <autoFilter ref="A1:P41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8795,7 +8467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -8834,7 +8506,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
     </row>
@@ -8846,7 +8518,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
     </row>
@@ -8891,7 +8563,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9">
@@ -8902,7 +8574,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>IRR #398 (OPEN/UNSTABLE); IPD none</t>
+          <t>IRR #398 merged during consolidated resolution; IPD none</t>
         </is>
       </c>
     </row>
@@ -9107,7 +8779,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Pending group: IPD implementation / deliverables</t>
+          <t>Pending group: IRR implementation / deliverables</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
@@ -9117,45 +8789,35 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Pending group: IRR implementation / deliverables</t>
+          <t>Pending group: Operator execution</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Pending group: Operator execution</t>
+          <t>Pending group: PA decisions / governance</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Pending group: PA decisions / governance</t>
+          <t>Pending group: Qualification / admission gates</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Pending group: Qualification / admission gates</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B31"/>
+  <autoFilter ref="A1:B30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9169,7 +8831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9225,7 +8887,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -9257,7 +8919,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -9267,12 +8929,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>tree 3e60d4f795a80e5656191947e792e8716dc2a031</t>
+          <t>tree 62785a3cdc099aab4090868629e745be9d1383e4</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Current authoritative IRR main; PR #397 merged; IRR-only CI 41195957176 success.</t>
+          <t>Current authoritative IRR main after PR #398; post-merge Windows run 41221317984 and static/recovery-audit run 41221318050 success.</t>
         </is>
       </c>
     </row>
@@ -9289,7 +8951,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9299,12 +8961,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>tree f12fd52d658bd8e8029106f77f4491b22b798485</t>
+          <t>tree e1e478ae3fad0ef02aeb85bf59d06ac0575cfed2</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Current authoritative IPD main; PR #113 merged; CI 41128431372 success.</t>
+          <t>Current authoritative IPD main after PR #114; CI 41219297374 success; code tree unchanged from 4e275ec9.</t>
         </is>
       </c>
     </row>
@@ -9321,7 +8983,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -9353,7 +9015,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -9363,12 +9025,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>31fd3b84746b7d47465f7cdf14e853c216ea71a5</t>
+          <t>5ceb5398b0cb172bdc793e62bdfaea005b7c426a</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>IPD execution tracker; final footer P-1 NOT AUTHORIZED is stale vs IRR P1-F and recorded as a conflict.</t>
+          <t>IPD execution tracker corrected by PR #114; stale P-1 NOT AUTHORIZED limb superseded by dated pointer; historical 31fd3b84 was a blob, not a commit.</t>
         </is>
       </c>
     </row>
@@ -9385,7 +9047,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -9417,7 +9079,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -9449,7 +9111,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -9481,7 +9143,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935 / 4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c / 527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -9513,7 +9175,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>e3dcb4dff1924bfc7a0c6046300ce7052fec6f3b</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -9523,12 +9185,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>OPEN / UNSTABLE</t>
+          <t>MERGED</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Unmerged consolidated P1/S2 correction; Windows PowerShell fixture run 41207888891 failure; static run 41207888919 success; proposes §16.230.</t>
+          <t>Consolidated P1/S2 correction merged; exact head eddbaead; Windows run 41220141777 and static/recovery-audit run 41220141940 PASS; post-merge runs 41221317984/41221318050 PASS; §16.230 and §16.232 preserved.</t>
         </is>
       </c>
     </row>
@@ -9545,7 +9207,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -9577,7 +9239,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -9609,7 +9271,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -9641,7 +9303,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935 / 4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c / 527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -9673,7 +9335,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -9705,7 +9367,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -9737,7 +9399,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -9769,7 +9431,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935 / 4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c / 527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -9801,7 +9463,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -9897,7 +9559,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -9929,7 +9591,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -9939,12 +9601,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>e94d2b801967fc50093f27177cd19276b51faf97</t>
+          <t>restamped 2026-10-31</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Runbook start path works; headline figures still 106/1350 while current head executes 108/1377; restamp pending.</t>
+          <t>Runbook start path preserved; headline figures restamped to 108 files / 1377 tests with exact frontend-tree verification pointer and raw receipts.</t>
         </is>
       </c>
     </row>
@@ -9961,7 +9623,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -9993,7 +9655,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -10025,7 +9687,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -10057,7 +9719,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -10089,7 +9751,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -10121,7 +9783,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -10153,7 +9815,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -10185,7 +9847,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -10217,7 +9879,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -10249,7 +9911,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -10281,7 +9943,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -10313,7 +9975,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>fff8cf98ddcc7af1c6ab58d3ae9a3442a5322935 / 4e275ec97a7701521e6a4e7632e9324bafe8d286</t>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c / 527f811b17edb02caa665b345d9f36102435e1e8</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -10364,8 +10026,200 @@
         </is>
       </c>
     </row>
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>E037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>evidence/integration/consolidated-outstanding-resolution-2026-10-31/</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>PR #398 merge read-back</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>17/17 PR #398 changed-path blobs independently read back at merge; script SHA-256 6639633855300cd645248ce597bb2c867b5cdbf6045947bf4281721bb1cde6d1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="60" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>E038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>IPD</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>527f811b17edb02caa665b345d9f36102435e1e8</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>evidence/integration/consolidated-outstanding-resolution-2026-10-31/raw/ipd-p20-verification.json</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>PR #114 remote verification</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>IPD PR #114 merged; one tracker path +90/-0; corrected blob 5ceb5398; main bytes match; CI 41219297374 success.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="60" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>E039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>evidence/integration/consolidated-outstanding-resolution-2026-10-31/raw/</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>108/1377 validation</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>npm ci/typecheck/replay/test:ci/guard/build PASS at frontend tree 67607e1d; S2-DEP-A rev-8 contract test corrected and focused 15/15 PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="60" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>E040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>docs/integration/IIPS_v3.0_CAP03_G14_DEPENDENCY_ASSESSMENT_2026-10-31.md</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>G14 dependency assessment</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>G2-G13 reconciled from current evidence; G14 final reconciliation BLOCKED/NOT STARTED because upstream gates remain incomplete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="60" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>E041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>IIPS_V3_E2E_MASTER_TRACKER_AND_IRR_IPD_DECISION_REGISTER_2026-10-13.md</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>§16.230/§16.231/§16.232 allocation census</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Headings unique; V1806-V1834 unique; CHG-09/10/11 reconciled; next free §16.233/CV-CORR-213/CHG-2026-10-31-12/V1835.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="60" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>E042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>7fd824de30d8268ed3eca210bc664dc60749fa8c</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>docs/integration/IIPS_v3.0_P20_IRR_PENDING_REGISTER_CLOSURE_2026-10-31.md</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>IRR P-20 closure</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>IRR pending register no longer lists the resolved IPD documentation conflict; IPD merge/blob references corrected; IRR/IPD ownership distinction preserved.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F37"/>
+  <autoFilter ref="A1:F43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -28896,7 +28750,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>

</xml_diff>